<commit_message>
deploy: production config, fix tsconfig, exclude magd_store
</commit_message>
<xml_diff>
--- a/backend/prisma/test.xlsx
+++ b/backend/prisma/test.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\123om\Downloads\cityyyaaa\backend\prisma\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\123om\Downloads\final-city-vol4\backend\prisma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00FD8DCE-3EDB-41C7-AA52-9B9404F69FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36FE2B1-5E4D-45DC-AB87-E71A74E82D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{F2D55117-9146-4D41-B952-A5B5286FD8D4}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{F2D55117-9146-4D41-B952-A5B5286FD8D4}"/>
   </bookViews>
   <sheets>
     <sheet name="TOTAL" sheetId="4" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2612" uniqueCount="1756">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2352" uniqueCount="1823">
   <si>
     <t>TOTAL</t>
   </si>
@@ -5311,6 +5311,207 @@
   </si>
   <si>
     <t>Quantity</t>
+  </si>
+  <si>
+    <t>طقم شنيور 98 قطعه</t>
+  </si>
+  <si>
+    <t>CK10-XA98</t>
+  </si>
+  <si>
+    <t>شنيور 810 وات</t>
+  </si>
+  <si>
+    <t>CT10130</t>
+  </si>
+  <si>
+    <t>CT10128</t>
+  </si>
+  <si>
+    <t>هيلتي عدل 800 وات BMC</t>
+  </si>
+  <si>
+    <t>CT18182</t>
+  </si>
+  <si>
+    <t>CT12041K</t>
+  </si>
+  <si>
+    <t>صاروخ قطعيه5"1010 وات</t>
+  </si>
+  <si>
+    <t>CT13023</t>
+  </si>
+  <si>
+    <t>صاروخ قطعيه 7بوصه 1300 وات</t>
+  </si>
+  <si>
+    <t>CT13044</t>
+  </si>
+  <si>
+    <t>صاروخ 9" 2200</t>
+  </si>
+  <si>
+    <t>ct13070</t>
+  </si>
+  <si>
+    <t>صاروخ 4.5 650 وات</t>
+  </si>
+  <si>
+    <t>CT13625</t>
+  </si>
+  <si>
+    <t>صاروخ 5" 710 وات</t>
+  </si>
+  <si>
+    <t>CT13649</t>
+  </si>
+  <si>
+    <t>اركت 550وات</t>
+  </si>
+  <si>
+    <t>CT15287</t>
+  </si>
+  <si>
+    <t>حليه الكتروني 8مم1050</t>
+  </si>
+  <si>
+    <t>CT11012</t>
+  </si>
+  <si>
+    <t>حليه الكتروني 12 مم 1850</t>
+  </si>
+  <si>
+    <t>CT11021</t>
+  </si>
+  <si>
+    <t>منشار صنيه 7 وربع 1500وات</t>
+  </si>
+  <si>
+    <t>ct15188_185</t>
+  </si>
+  <si>
+    <t>صنفره هزاز 90مم230مم200</t>
+  </si>
+  <si>
+    <t>CT13562</t>
+  </si>
+  <si>
+    <t>مفك عاده صيني 38*6</t>
+  </si>
+  <si>
+    <t>CPHDS-AS0603</t>
+  </si>
+  <si>
+    <t>قشاره سلك 6"</t>
+  </si>
+  <si>
+    <t>CPHEP_WSA06</t>
+  </si>
+  <si>
+    <t>مفتاح فرنساوي 10 صيني</t>
+  </si>
+  <si>
+    <t>CPHWA_CNA10</t>
+  </si>
+  <si>
+    <t>مفتاح فرنساوي 12صيني</t>
+  </si>
+  <si>
+    <t>CPHWA_CNA12</t>
+  </si>
+  <si>
+    <t>CPHWA_CNA08</t>
+  </si>
+  <si>
+    <t>بنسه كلابه بوز عدل 10 صيني</t>
+  </si>
+  <si>
+    <t>CPHPL_GSB10</t>
+  </si>
+  <si>
+    <t>CPHPL_RTA10</t>
+  </si>
+  <si>
+    <t>طقم عدد يدوي 14 قطعه شنطه</t>
+  </si>
+  <si>
+    <t>CPHTS-BXA14</t>
+  </si>
+  <si>
+    <t>طقم الن هكس اكثر طولا 9 قطع</t>
+  </si>
+  <si>
+    <t>CPHOK-HMCX09</t>
+  </si>
+  <si>
+    <t>برواز منشار حدادي 12 بوصه</t>
+  </si>
+  <si>
+    <t>CPHSH_FXA12</t>
+  </si>
+  <si>
+    <t>مفتاح عجل صليبه مقاس 17*14*13*12</t>
+  </si>
+  <si>
+    <t>مقص صاج شمال 10 صيني</t>
+  </si>
+  <si>
+    <t>CPHSSD_CLA10</t>
+  </si>
+  <si>
+    <t>مقص مواسير 42صيني</t>
+  </si>
+  <si>
+    <t>CPHSC_PCA42</t>
+  </si>
+  <si>
+    <t>مقص صاج عدل 10 صيني</t>
+  </si>
+  <si>
+    <t>CPHSSD_CSA10</t>
+  </si>
+  <si>
+    <t>مقص صاج يمين 10 صيني</t>
+  </si>
+  <si>
+    <t>CPHSSD_CRA10</t>
+  </si>
+  <si>
+    <t>بنطه 4مم اتجاهين</t>
+  </si>
+  <si>
+    <t>CTHDP0101</t>
+  </si>
+  <si>
+    <t>مقص فواكه 8"</t>
+  </si>
+  <si>
+    <t>CPHSS-PRA08</t>
+  </si>
+  <si>
+    <t>متر ليز 60</t>
+  </si>
+  <si>
+    <t>CT44029</t>
+  </si>
+  <si>
+    <t>ميزان ليز 2 خط 15 متر</t>
+  </si>
+  <si>
+    <t>CT44046</t>
+  </si>
+  <si>
+    <t>حامل ميزان ليزر</t>
+  </si>
+  <si>
+    <t>CAXL-S12</t>
+  </si>
+  <si>
+    <t>جهاز قياس كلامب ميتر امبير</t>
+  </si>
+  <si>
+    <t>CT44053</t>
   </si>
 </sst>
 </file>
@@ -19806,7 +20007,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0B1D24D-ABB3-4215-8065-2ACEB70148E9}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:H260"/>
+  <dimension ref="A1:H127"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="18.75" outlineLevelRow="1" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="2" customWidth="1"/>
@@ -19815,8 +20016,7 @@
     <col min="4" max="4" width="56.28515625" style="2" bestFit="1" customWidth="1" outlineLevel="1"/>
     <col min="5" max="5" width="17" style="2" customWidth="1" outlineLevel="1"/>
     <col min="6" max="6" width="24.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="28.7109375" style="2" customWidth="1"/>
+    <col min="7" max="8" width="8.85546875" style="2"/>
     <col min="9" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
@@ -19865,3205 +20065,1031 @@
     </row>
     <row r="5" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D5" s="2" t="s">
-        <v>1219</v>
+        <v>1756</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1220</v>
-      </c>
-      <c r="F5" s="7">
-        <v>6221257437829</v>
+        <v>1757</v>
+      </c>
+      <c r="F5" s="7"/>
+      <c r="G5" s="2">
+        <v>1653</v>
       </c>
       <c r="H5" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D6" s="2" t="s">
-        <v>1223</v>
+        <v>1758</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1224</v>
-      </c>
-      <c r="F6" s="7">
-        <v>6221257353211</v>
-      </c>
+        <v>1759</v>
+      </c>
+      <c r="F6" s="7"/>
       <c r="G6" s="2">
-        <v>701</v>
+        <v>1552</v>
       </c>
       <c r="H6" s="2">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D7" s="2" t="s">
-        <v>1225</v>
+        <v>1129</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1226</v>
-      </c>
-      <c r="F7" s="7">
-        <v>6223007700030</v>
-      </c>
+        <v>1760</v>
+      </c>
+      <c r="F7" s="7"/>
       <c r="G7" s="2">
-        <v>770</v>
+        <v>807</v>
       </c>
       <c r="H7" s="2">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D8" s="2" t="s">
-        <v>1221</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>1222</v>
-      </c>
-      <c r="F8" s="8">
-        <v>6221257527612</v>
-      </c>
-      <c r="G8" s="2">
-        <v>2257</v>
-      </c>
-      <c r="H8" s="2">
-        <v>6</v>
-      </c>
+      <c r="C8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="8"/>
     </row>
     <row r="9" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C9" s="2" t="s">
-        <v>55</v>
+      <c r="D9" s="2" t="s">
+        <v>1761</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>1762</v>
       </c>
       <c r="F9" s="8"/>
+      <c r="G9" s="2">
+        <v>2263</v>
+      </c>
+      <c r="H9" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D10" s="2" t="s">
-        <v>1227</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>1228</v>
-      </c>
-      <c r="F10" s="8">
-        <v>6221257353365</v>
-      </c>
-      <c r="G10" s="2">
-        <v>1902</v>
-      </c>
-      <c r="H10" s="2">
-        <v>11</v>
-      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="8"/>
     </row>
     <row r="11" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D11" s="2" t="s">
-        <v>1229</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>1230</v>
-      </c>
-      <c r="F11" s="8">
-        <v>6221257507935</v>
-      </c>
-      <c r="G11" s="2">
-        <v>5843</v>
-      </c>
-      <c r="H11" s="2">
-        <v>1</v>
-      </c>
+      <c r="C11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="8"/>
     </row>
     <row r="12" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D12" s="2" t="s">
-        <v>1231</v>
+        <v>956</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1232</v>
+        <v>1763</v>
       </c>
       <c r="F12" s="8"/>
       <c r="G12" s="2">
-        <v>5964</v>
+        <v>696</v>
       </c>
       <c r="H12" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D13" s="2" t="s">
-        <v>1233</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>1234</v>
+      <c r="C13" s="2" t="s">
+        <v>264</v>
       </c>
       <c r="F13" s="8"/>
-      <c r="G13" s="2">
-        <v>2832</v>
-      </c>
-      <c r="H13" s="2">
-        <v>0</v>
-      </c>
     </row>
     <row r="14" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D14" s="2" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>1236</v>
-      </c>
-      <c r="F14" s="8">
-        <v>6223007700061</v>
-      </c>
-      <c r="G14" s="2">
-        <v>1858</v>
-      </c>
-      <c r="H14" s="2">
-        <v>7</v>
-      </c>
+      <c r="C14" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F14" s="8"/>
     </row>
     <row r="15" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D15" s="2" t="s">
-        <v>1237</v>
+        <v>1764</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>1238</v>
+        <v>1765</v>
       </c>
       <c r="F15" s="8"/>
       <c r="G15" s="2">
-        <v>1708</v>
+        <v>1291</v>
       </c>
       <c r="H15" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D16" s="2" t="s">
-        <v>1239</v>
+        <v>1766</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>1240</v>
+        <v>1767</v>
       </c>
       <c r="F16" s="8"/>
       <c r="G16" s="2">
-        <v>2534</v>
+        <v>1881</v>
       </c>
       <c r="H16" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D17" s="2" t="s">
-        <v>1241</v>
+        <v>1768</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>1242</v>
-      </c>
-      <c r="F17" s="8">
-        <v>6221257507911</v>
-      </c>
+        <v>1769</v>
+      </c>
+      <c r="F17" s="8"/>
       <c r="G17" s="2">
-        <v>2878</v>
+        <v>2448</v>
       </c>
       <c r="H17" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D18" s="2" t="s">
-        <v>1254</v>
+        <v>1770</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1255</v>
-      </c>
-      <c r="F18" s="8">
-        <v>6221257353419</v>
-      </c>
+        <v>1771</v>
+      </c>
+      <c r="F18" s="8"/>
       <c r="G18" s="2">
-        <v>2560</v>
+        <v>825</v>
       </c>
       <c r="H18" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="8"/>
+      <c r="D19" s="2" t="s">
+        <v>1772</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>1773</v>
+      </c>
+      <c r="F19" s="8">
+        <v>7640228053537</v>
+      </c>
+      <c r="G19" s="2">
+        <v>1178</v>
+      </c>
+      <c r="H19" s="2">
+        <v>6</v>
+      </c>
     </row>
     <row r="20" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D20" s="2" t="s">
-        <v>1267</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>1268</v>
-      </c>
-      <c r="F20" s="8">
-        <v>6221257520712</v>
-      </c>
-      <c r="G20" s="2">
-        <v>547</v>
-      </c>
-      <c r="H20" s="2">
-        <v>2</v>
-      </c>
+      <c r="C20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F20" s="8"/>
     </row>
     <row r="21" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="2" t="s">
-        <v>60</v>
+      <c r="D21" s="2" t="s">
+        <v>1774</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>1775</v>
       </c>
       <c r="F21" s="8"/>
+      <c r="G21" s="2">
+        <v>1196</v>
+      </c>
+      <c r="H21" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D22" s="2" t="s">
-        <v>956</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>1247</v>
+      <c r="C22" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="F22" s="8"/>
-      <c r="G22" s="2">
-        <v>615</v>
-      </c>
-      <c r="H22" s="2">
-        <v>5</v>
-      </c>
     </row>
     <row r="23" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D23" s="2" t="s">
-        <v>1065</v>
+        <v>1776</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>1293</v>
-      </c>
-      <c r="F23" s="8">
-        <v>6221257354027</v>
-      </c>
+        <v>1777</v>
+      </c>
+      <c r="F23" s="8"/>
       <c r="G23" s="2">
-        <v>615</v>
+        <v>2351</v>
       </c>
       <c r="H23" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="3:8" ht="17.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D24" s="2" t="s">
-        <v>1294</v>
+        <v>1778</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1295</v>
-      </c>
-      <c r="F24" s="8">
-        <v>6221257520743</v>
-      </c>
+        <v>1779</v>
+      </c>
+      <c r="F24" s="8"/>
       <c r="G24" s="2">
-        <v>526</v>
+        <v>2755</v>
       </c>
       <c r="H24" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C25" s="2" t="s">
-        <v>264</v>
+        <v>9</v>
       </c>
       <c r="F25" s="8"/>
     </row>
     <row r="26" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C26" s="2" t="s">
-        <v>6</v>
+      <c r="D26" s="2" t="s">
+        <v>1780</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>1781</v>
       </c>
       <c r="F26" s="8"/>
+      <c r="G26" s="2">
+        <v>2417</v>
+      </c>
+      <c r="H26" s="2">
+        <v>1</v>
+      </c>
     </row>
     <row r="27" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D27" s="2" t="s">
-        <v>1243</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>1244</v>
+      <c r="C27" s="2" t="s">
+        <v>10</v>
       </c>
       <c r="F27" s="8"/>
-      <c r="G27" s="2">
-        <v>2198</v>
-      </c>
-      <c r="H27" s="2">
-        <v>6</v>
-      </c>
     </row>
     <row r="28" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D28" s="2" t="s">
-        <v>1120</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>1256</v>
-      </c>
-      <c r="F28" s="8">
-        <v>6221257353655</v>
-      </c>
-      <c r="G28" s="2">
-        <v>2570</v>
-      </c>
-      <c r="H28" s="2">
-        <v>0</v>
-      </c>
+      <c r="C28" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28" s="8"/>
     </row>
     <row r="29" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D29" s="2" t="s">
-        <v>1257</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>1258</v>
-      </c>
-      <c r="F29" s="8">
-        <v>6221257513967</v>
-      </c>
-      <c r="G29" s="2">
-        <v>865</v>
-      </c>
-      <c r="H29" s="2">
-        <v>6</v>
-      </c>
+      <c r="C29" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F29" s="8"/>
     </row>
     <row r="30" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D30" s="2" t="s">
-        <v>1259</v>
+        <v>1782</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>1260</v>
+        <v>1783</v>
       </c>
       <c r="F30" s="8"/>
       <c r="G30" s="2">
-        <v>853</v>
+        <v>932</v>
       </c>
       <c r="H30" s="2">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D31" s="2" t="s">
-        <v>1261</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>1262</v>
-      </c>
-      <c r="F31" s="8">
-        <v>6221257456127</v>
-      </c>
-      <c r="G31" s="2">
-        <v>1227</v>
-      </c>
-      <c r="H31" s="2">
-        <v>12</v>
-      </c>
+      <c r="C31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" s="8"/>
     </row>
     <row r="32" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D32" s="2" t="s">
-        <v>1263</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>1264</v>
+      <c r="C32" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="F32" s="8"/>
-      <c r="G32" s="2">
-        <v>2079</v>
-      </c>
-      <c r="H32" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D33" s="2" t="s">
-        <v>1265</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>1266</v>
-      </c>
-      <c r="F33" s="8">
-        <v>6221257353631</v>
-      </c>
-      <c r="G33" s="2">
-        <v>1725</v>
-      </c>
-      <c r="H33" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D34" s="2" t="s">
-        <v>1277</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>1278</v>
-      </c>
-      <c r="F34" s="8">
-        <v>6221257526684</v>
-      </c>
-      <c r="G34" s="2">
-        <v>1602</v>
-      </c>
-      <c r="H34" s="2">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="35" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D35" s="2" t="s">
-        <v>1279</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>1280</v>
-      </c>
-      <c r="F35" s="8">
-        <v>6221257541229</v>
-      </c>
-      <c r="G35" s="2">
-        <v>1881</v>
-      </c>
-      <c r="H35" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D36" s="2" t="s">
-        <v>1245</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>1246</v>
+    </row>
+    <row r="33" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C33" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F33" s="8"/>
+    </row>
+    <row r="34" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C34" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F34" s="8"/>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B35" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" s="8"/>
+    </row>
+    <row r="36" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C36" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="F36" s="8"/>
-      <c r="G36" s="2">
-        <v>1083</v>
-      </c>
-      <c r="H36" s="2">
+    </row>
+    <row r="37" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D37" s="2" t="s">
+        <v>1784</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>1785</v>
+      </c>
+      <c r="F37" s="8"/>
+      <c r="G37" s="2">
+        <v>34</v>
+      </c>
+      <c r="H37" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C37" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F37" s="8"/>
-    </row>
-    <row r="38" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D38" s="2" t="s">
-        <v>1269</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>1270</v>
-      </c>
-      <c r="F38" s="8">
-        <v>6221257353785</v>
-      </c>
-      <c r="G38" s="2">
-        <v>1274</v>
-      </c>
-      <c r="H38" s="2">
+    <row r="38" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C38" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="F38" s="8"/>
+    </row>
+    <row r="39" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C39" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F39" s="8"/>
+    </row>
+    <row r="40" spans="2:8" ht="19.5" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C40" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F40" s="8"/>
+    </row>
+    <row r="41" spans="2:8" ht="19.5" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D41" s="4" t="s">
+        <v>1786</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>1787</v>
+      </c>
+      <c r="F41" s="8"/>
+      <c r="G41" s="4">
+        <v>110</v>
+      </c>
+      <c r="H41" s="13">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D39" s="2" t="s">
-        <v>1271</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>1272</v>
-      </c>
-      <c r="F39" s="8">
-        <v>6221257353778</v>
-      </c>
-      <c r="G39" s="2">
-        <v>1010</v>
-      </c>
-      <c r="H39" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D40" s="2" t="s">
-        <v>1273</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>1274</v>
-      </c>
-      <c r="F40" s="8">
-        <v>6221257523812</v>
-      </c>
-      <c r="G40" s="2">
-        <v>747</v>
-      </c>
-      <c r="H40" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="41" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C41" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F41" s="8"/>
-    </row>
-    <row r="42" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D42" s="2" t="s">
-        <v>1480</v>
+        <v>1788</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>1481</v>
-      </c>
-      <c r="F42" s="8">
-        <v>6221257353792</v>
-      </c>
+        <v>1789</v>
+      </c>
+      <c r="F42" s="8"/>
       <c r="G42" s="2">
-        <v>1034</v>
+        <v>153</v>
       </c>
       <c r="H42" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C43" s="2" t="s">
-        <v>9</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D43" s="2" t="s">
+        <v>1790</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>1791</v>
       </c>
       <c r="F43" s="8"/>
-    </row>
-    <row r="44" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="G43" s="2">
+        <v>222</v>
+      </c>
+      <c r="H43" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D44" s="2" t="s">
-        <v>1275</v>
+        <v>578</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>1276</v>
-      </c>
-      <c r="F44" s="8">
-        <v>6221257353723</v>
-      </c>
+        <v>1792</v>
+      </c>
+      <c r="F44" s="8"/>
       <c r="G44" s="2">
-        <v>1927</v>
+        <v>111</v>
       </c>
       <c r="H44" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="45" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D45" s="2" t="s">
-        <v>1284</v>
+        <v>1793</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>1285</v>
-      </c>
-      <c r="F45" s="8">
-        <v>6221257456271</v>
-      </c>
+        <v>1794</v>
+      </c>
+      <c r="F45" s="8"/>
       <c r="G45" s="2">
-        <v>2460</v>
+        <v>121</v>
       </c>
       <c r="H45" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="46" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C46" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D46" s="2" t="s">
+        <v>843</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>1795</v>
       </c>
       <c r="F46" s="8"/>
-    </row>
-    <row r="47" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D47" s="2" t="s">
-        <v>1248</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>1249</v>
+      <c r="G46" s="2">
+        <v>122</v>
+      </c>
+      <c r="H46" s="2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C47" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="F47" s="8"/>
-      <c r="G47" s="2">
-        <v>2422</v>
-      </c>
-      <c r="H47" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="48" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D48" s="2" t="s">
-        <v>1250</v>
+        <v>1796</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>1251</v>
+        <v>1797</v>
       </c>
       <c r="F48" s="8"/>
       <c r="G48" s="2">
-        <v>2939</v>
+        <v>685</v>
       </c>
       <c r="H48" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D49" s="2" t="s">
-        <v>1281</v>
-      </c>
-      <c r="E49" s="2" t="s">
-        <v>1282</v>
+    <row r="49" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C49" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="F49" s="8"/>
-      <c r="G49" s="2">
-        <v>6267</v>
-      </c>
-      <c r="H49" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D50" s="2" t="s">
-        <v>1283</v>
-      </c>
-      <c r="E50" s="2" t="s">
-        <v>1251</v>
-      </c>
-      <c r="F50" s="8">
-        <v>6221257353860</v>
-      </c>
-      <c r="G50" s="2">
-        <v>2939</v>
-      </c>
-      <c r="H50" s="2">
+    </row>
+    <row r="50" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C50" s="2" t="s">
+        <v>881</v>
+      </c>
+      <c r="F50" s="8"/>
+    </row>
+    <row r="51" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D51" s="2" t="s">
+        <v>1798</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>1799</v>
+      </c>
+      <c r="F51" s="8"/>
+      <c r="G51" s="2">
+        <v>135</v>
+      </c>
+      <c r="H51" s="2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C52" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F52" s="8"/>
+    </row>
+    <row r="53" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C53" s="2" t="s">
+        <v>682</v>
+      </c>
+      <c r="F53" s="8"/>
+    </row>
+    <row r="54" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C54" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F54" s="8"/>
+    </row>
+    <row r="55" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C55" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="F55" s="8"/>
+    </row>
+    <row r="56" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C56" s="2" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F56" s="8"/>
+    </row>
+    <row r="57" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C57" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F57" s="8"/>
+    </row>
+    <row r="58" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D58" s="2" t="s">
+        <v>1800</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>1801</v>
+      </c>
+      <c r="F58" s="8"/>
+      <c r="G58" s="2">
+        <v>130</v>
+      </c>
+      <c r="H58" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D51" s="2" t="s">
-        <v>1286</v>
-      </c>
-      <c r="E51" s="2" t="s">
-        <v>1249</v>
-      </c>
-      <c r="F51" s="8">
-        <v>6221257377149</v>
-      </c>
-      <c r="G51" s="2">
-        <v>2422</v>
-      </c>
-      <c r="H51" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D52" s="2" t="s">
-        <v>1287</v>
-      </c>
-      <c r="E52" s="2" t="s">
-        <v>1288</v>
-      </c>
-      <c r="F52" s="8">
-        <v>6221257353877</v>
-      </c>
-      <c r="H52" s="2">
+    <row r="59" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C59" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F59" s="8"/>
+    </row>
+    <row r="60" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C60" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F60" s="8"/>
+    </row>
+    <row r="61" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C61" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F61" s="8"/>
+    </row>
+    <row r="62" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C62" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F62" s="8"/>
+    </row>
+    <row r="63" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C63" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="F63" s="8"/>
+    </row>
+    <row r="64" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C64" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F64" s="8"/>
+    </row>
+    <row r="65" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D65" s="2" t="s">
+        <v>1802</v>
+      </c>
+      <c r="F65" s="8"/>
+      <c r="G65" s="2">
+        <v>96</v>
+      </c>
+      <c r="H65" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="66" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C66" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F66" s="8"/>
+    </row>
+    <row r="67" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C67" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F67" s="8"/>
+    </row>
+    <row r="68" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D68" s="2" t="s">
+        <v>1803</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>1804</v>
+      </c>
+      <c r="F68" s="8"/>
+      <c r="G68" s="2">
+        <v>130</v>
+      </c>
+      <c r="H68" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C53" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F53" s="8"/>
-    </row>
-    <row r="54" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D54" s="2" t="s">
-        <v>1445</v>
-      </c>
-      <c r="E54" s="2" t="s">
-        <v>1446</v>
-      </c>
-      <c r="F54" s="8">
-        <v>6221257353747</v>
-      </c>
-      <c r="G54" s="2">
-        <v>1480</v>
-      </c>
-      <c r="H54" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C55" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F55" s="8"/>
-    </row>
-    <row r="56" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D56" s="2" t="s">
-        <v>1411</v>
-      </c>
-      <c r="E56" s="2" t="s">
-        <v>1412</v>
-      </c>
-      <c r="F56" s="8">
-        <v>6221257030716</v>
-      </c>
-      <c r="G56" s="2">
-        <v>35</v>
-      </c>
-      <c r="H56" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="57" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D57" s="2" t="s">
-        <v>1501</v>
-      </c>
-      <c r="E57" s="2" t="s">
-        <v>1502</v>
-      </c>
-      <c r="F57" s="8">
-        <v>6221257523782</v>
-      </c>
-      <c r="G57" s="2">
-        <v>709</v>
-      </c>
-      <c r="H57" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="58" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D58" s="2" t="s">
-        <v>1503</v>
-      </c>
-      <c r="E58" s="2" t="s">
-        <v>1504</v>
-      </c>
-      <c r="F58" s="8">
-        <v>6221257523799</v>
-      </c>
-      <c r="G58" s="2">
-        <v>895</v>
-      </c>
-      <c r="H58" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="59" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C59" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F59" s="8"/>
-    </row>
-    <row r="60" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C60" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F60" s="8"/>
-    </row>
-    <row r="61" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C61" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F61" s="8"/>
-    </row>
-    <row r="62" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D62" s="2" t="s">
-        <v>1289</v>
-      </c>
-      <c r="E62" s="2" t="s">
-        <v>1290</v>
-      </c>
-      <c r="F62" s="8"/>
-      <c r="G62" s="2">
-        <v>1459</v>
-      </c>
-      <c r="H62" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C63" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F63" s="8"/>
-    </row>
-    <row r="64" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B64" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F64" s="8"/>
-    </row>
-    <row r="65" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C65" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F65" s="8"/>
-    </row>
-    <row r="66" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D66" s="2" t="s">
-        <v>1378</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>1379</v>
-      </c>
-      <c r="F66" s="8">
-        <v>6221257375695</v>
-      </c>
-      <c r="G66" s="2">
-        <v>47</v>
-      </c>
-      <c r="H66" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="67" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D67" s="2" t="s">
-        <v>1380</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>1381</v>
-      </c>
-      <c r="F67" s="8">
-        <v>79011000161</v>
-      </c>
-      <c r="H67" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D68" s="2" t="s">
-        <v>1382</v>
-      </c>
-      <c r="E68" s="2" t="s">
-        <v>1383</v>
-      </c>
-      <c r="F68" s="8">
-        <v>6221257484977</v>
-      </c>
-      <c r="G68" s="2">
-        <v>15</v>
-      </c>
-      <c r="H68" s="2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="69" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D69" s="2" t="s">
-        <v>1384</v>
+        <v>1805</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>1385</v>
-      </c>
-      <c r="F69" s="8">
-        <v>6221257487787</v>
-      </c>
+        <v>1806</v>
+      </c>
+      <c r="F69" s="8"/>
       <c r="G69" s="2">
-        <v>19</v>
+        <v>120</v>
       </c>
       <c r="H69" s="2">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="70" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D70" s="2" t="s">
-        <v>1386</v>
+        <v>1807</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>1387</v>
+        <v>1808</v>
       </c>
       <c r="F70" s="8"/>
       <c r="G70" s="2">
-        <v>21</v>
+        <v>130</v>
       </c>
       <c r="H70" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="71" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="71" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D71" s="2" t="s">
-        <v>1388</v>
+        <v>1809</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>1389</v>
+        <v>1810</v>
       </c>
       <c r="F71" s="8"/>
       <c r="G71" s="2">
-        <v>23</v>
+        <v>130</v>
       </c>
       <c r="H71" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="72" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C72" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F72" s="8"/>
+    </row>
+    <row r="73" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C73" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F73" s="8"/>
+    </row>
+    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B74" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F74" s="8"/>
+    </row>
+    <row r="75" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C75" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F75" s="8"/>
+    </row>
+    <row r="76" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="D76" s="2" t="s">
+        <v>1811</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>1812</v>
+      </c>
+      <c r="F76" s="8"/>
+      <c r="H76" s="2">
         <v>20</v>
       </c>
     </row>
-    <row r="72" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D72" s="2" t="s">
-        <v>1390</v>
-      </c>
-      <c r="E72" s="2" t="s">
-        <v>1391</v>
-      </c>
-      <c r="F72" s="8">
-        <v>6221257484281</v>
-      </c>
-      <c r="G72" s="2">
-        <v>15</v>
-      </c>
-      <c r="H72" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="73" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D73" s="2" t="s">
-        <v>1392</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>1393</v>
-      </c>
-      <c r="F73" s="8"/>
-      <c r="G73" s="2">
-        <v>100</v>
-      </c>
-      <c r="H73" s="2">
+    <row r="77" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C77" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F77" s="8"/>
+    </row>
+    <row r="78" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C78" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F78" s="8"/>
+    </row>
+    <row r="79" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C79" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="F79" s="8"/>
+    </row>
+    <row r="80" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C80" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F80" s="8"/>
+    </row>
+    <row r="81" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C81" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F81" s="8"/>
+    </row>
+    <row r="82" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C82" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F82" s="8"/>
+    </row>
+    <row r="83" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B83" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F83" s="8"/>
+    </row>
+    <row r="84" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C84" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F84" s="8"/>
+    </row>
+    <row r="85" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C85" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F85" s="8"/>
+    </row>
+    <row r="86" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C86" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F86" s="8"/>
+    </row>
+    <row r="87" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C87" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" s="8"/>
+    </row>
+    <row r="88" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C88" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="F88" s="8"/>
+    </row>
+    <row r="89" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C89" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F89" s="8"/>
+    </row>
+    <row r="90" spans="2:8" ht="17.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C90" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="74" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D74" s="2" t="s">
-        <v>1394</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>1395</v>
-      </c>
-      <c r="F74" s="8">
-        <v>6221257484311</v>
-      </c>
-      <c r="G74" s="2">
-        <v>18</v>
-      </c>
-      <c r="H74" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="75" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D75" s="2" t="s">
-        <v>1396</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>1397</v>
-      </c>
-      <c r="F75" s="8">
-        <v>6223007701761</v>
-      </c>
-      <c r="G75" s="2">
-        <v>29</v>
-      </c>
-      <c r="H75" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="76" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D76" s="2" t="s">
-        <v>1398</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>1399</v>
-      </c>
-      <c r="F76" s="8"/>
-      <c r="G76" s="2">
-        <v>35</v>
-      </c>
-      <c r="H76" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D77" s="2" t="s">
-        <v>1400</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>1401</v>
-      </c>
-      <c r="F77" s="8">
-        <v>6223007702980</v>
-      </c>
-      <c r="G77" s="2">
-        <v>50</v>
-      </c>
-      <c r="H77" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="78" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D78" s="2" t="s">
-        <v>1402</v>
-      </c>
-      <c r="E78" s="2">
-        <v>506025</v>
-      </c>
-      <c r="F78" s="8"/>
-      <c r="G78" s="2">
-        <v>106</v>
-      </c>
-      <c r="H78" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="79" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D79" s="2" t="s">
-        <v>1403</v>
-      </c>
-      <c r="E79" s="2">
-        <v>506002</v>
-      </c>
-      <c r="F79" s="8"/>
-      <c r="G79" s="2">
-        <v>58</v>
-      </c>
-      <c r="H79" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D80" s="2" t="s">
-        <v>1404</v>
-      </c>
-      <c r="E80" s="2">
-        <v>506005</v>
-      </c>
-      <c r="F80" s="8"/>
-      <c r="G80" s="2">
-        <v>100</v>
-      </c>
-      <c r="H80" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="81" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D81" s="2" t="s">
-        <v>1413</v>
-      </c>
-      <c r="E81" s="2" t="s">
-        <v>1414</v>
-      </c>
-      <c r="F81" s="8"/>
-      <c r="G81" s="2">
-        <v>103</v>
-      </c>
-      <c r="H81" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C82" s="2" t="s">
-        <v>636</v>
-      </c>
-      <c r="F82" s="8"/>
-    </row>
-    <row r="83" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C83" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="F83" s="8"/>
-    </row>
-    <row r="84" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D84" s="2" t="s">
-        <v>1461</v>
-      </c>
-      <c r="E84" s="2">
-        <v>123012</v>
-      </c>
-      <c r="F84" s="8"/>
-      <c r="G84" s="2">
-        <v>731</v>
-      </c>
-      <c r="H84" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="85" spans="3:8" ht="19.5" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C85" s="11" t="s">
-        <v>99</v>
-      </c>
-      <c r="F85" s="8"/>
-    </row>
-    <row r="86" spans="3:8" ht="19.5" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D86" s="4" t="s">
-        <v>1351</v>
-      </c>
-      <c r="E86" s="9" t="s">
-        <v>1352</v>
-      </c>
-      <c r="F86" s="8"/>
-      <c r="G86" s="4">
-        <v>76</v>
-      </c>
-      <c r="H86" s="13">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="87" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D87" s="2" t="s">
-        <v>1353</v>
-      </c>
-      <c r="E87" s="2" t="s">
-        <v>1354</v>
-      </c>
-      <c r="F87" s="8"/>
-      <c r="H87" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D88" s="2" t="s">
-        <v>1355</v>
-      </c>
-      <c r="E88" s="2" t="s">
-        <v>1356</v>
-      </c>
-      <c r="F88" s="8"/>
-      <c r="G88" s="2">
-        <v>135</v>
-      </c>
-      <c r="H88" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="89" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D89" s="2" t="s">
-        <v>1357</v>
-      </c>
-      <c r="E89" s="2" t="s">
-        <v>1358</v>
-      </c>
-      <c r="F89" s="8">
-        <v>6223007708883</v>
-      </c>
-      <c r="G89" s="2">
-        <v>130</v>
-      </c>
-      <c r="H89" s="2">
+      <c r="F90" s="8"/>
+    </row>
+    <row r="91" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B91" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="90" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D90" s="2" t="s">
-        <v>1359</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>1360</v>
-      </c>
-      <c r="F90" s="8">
-        <v>6221257496451</v>
-      </c>
-      <c r="G90" s="2">
-        <v>66</v>
-      </c>
-      <c r="H90" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="91" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D91" s="2" t="s">
-        <v>1361</v>
-      </c>
-      <c r="E91" s="2" t="s">
-        <v>1362</v>
-      </c>
-      <c r="F91" s="8">
-        <v>6221257496468</v>
-      </c>
-      <c r="G91" s="2">
-        <v>80</v>
-      </c>
-      <c r="H91" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="92" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D92" s="2" t="s">
-        <v>1363</v>
-      </c>
-      <c r="E92" s="2" t="s">
-        <v>1364</v>
-      </c>
-      <c r="F92" s="8">
-        <v>6223007708920</v>
-      </c>
-      <c r="G92" s="2">
-        <v>136</v>
-      </c>
-      <c r="H92" s="2">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="93" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D93" s="2" t="s">
-        <v>616</v>
-      </c>
-      <c r="E93" s="2" t="s">
-        <v>1365</v>
-      </c>
-      <c r="F93" s="8">
-        <v>6223007708937</v>
-      </c>
-      <c r="G93" s="2">
-        <v>136</v>
-      </c>
-      <c r="H93" s="2">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="94" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D94" s="2" t="s">
-        <v>1447</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>1448</v>
+      <c r="F91" s="8"/>
+    </row>
+    <row r="92" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C92" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F92" s="8"/>
+    </row>
+    <row r="93" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C93" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F93" s="8"/>
+    </row>
+    <row r="94" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C94" s="2" t="s">
+        <v>48</v>
       </c>
       <c r="F94" s="8"/>
-      <c r="G94" s="2">
-        <v>220</v>
-      </c>
-      <c r="H94" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="95" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D95" s="2" t="s">
-        <v>1449</v>
+        <v>1813</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>1450</v>
+        <v>1814</v>
       </c>
       <c r="F95" s="8"/>
       <c r="G95" s="2">
-        <v>262</v>
+        <v>106</v>
       </c>
       <c r="H95" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="96" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D96" s="2" t="s">
-        <v>1451</v>
-      </c>
-      <c r="E96" s="2" t="s">
-        <v>1452</v>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="96" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C96" s="2" t="s">
+        <v>521</v>
       </c>
       <c r="F96" s="8"/>
-      <c r="G96" s="2">
-        <v>396</v>
-      </c>
-      <c r="H96" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D97" s="2" t="s">
-        <v>1464</v>
-      </c>
-      <c r="E97" s="2" t="s">
-        <v>1465</v>
+    </row>
+    <row r="97" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C97" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="F97" s="8"/>
-      <c r="G97" s="2">
-        <v>150</v>
-      </c>
-      <c r="H97" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="98" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D98" s="2" t="s">
-        <v>1466</v>
-      </c>
-      <c r="E98" s="2" t="s">
-        <v>1467</v>
-      </c>
-      <c r="F98" s="8">
-        <v>6223007702669</v>
-      </c>
-      <c r="G98" s="2">
-        <v>180</v>
-      </c>
-      <c r="H98" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="99" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D99" s="2" t="s">
-        <v>1468</v>
-      </c>
-      <c r="E99" s="2" t="s">
-        <v>1469</v>
-      </c>
-      <c r="F99" s="8">
-        <v>6221257378771</v>
-      </c>
-      <c r="G99" s="2">
-        <v>177</v>
-      </c>
-      <c r="H99" s="2">
+    </row>
+    <row r="98" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C98" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F98" s="8"/>
+    </row>
+    <row r="99" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C99" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F99" s="8"/>
+    </row>
+    <row r="100" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B100" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="100" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D100" s="2" t="s">
-        <v>1470</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>1471</v>
-      </c>
-      <c r="F100" s="8">
-        <v>6221257378764</v>
-      </c>
-      <c r="G100" s="2">
-        <v>155</v>
-      </c>
-      <c r="H100" s="2">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="101" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D101" s="2" t="s">
-        <v>1472</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>1473</v>
+      <c r="F100" s="8"/>
+    </row>
+    <row r="101" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C101" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="F101" s="8"/>
-      <c r="G101" s="2">
-        <v>76</v>
-      </c>
-      <c r="H101" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="102" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D102" s="2" t="s">
-        <v>1474</v>
-      </c>
-      <c r="E102" s="2" t="s">
-        <v>1475</v>
-      </c>
-      <c r="F102" s="8">
-        <v>6221257482027</v>
-      </c>
-      <c r="G102" s="2">
-        <v>76</v>
-      </c>
-      <c r="H102" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="103" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="102" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C102" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F102" s="8"/>
+    </row>
+    <row r="103" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D103" s="2" t="s">
-        <v>1525</v>
+        <v>1815</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>1526</v>
+        <v>1816</v>
       </c>
       <c r="F103" s="8"/>
       <c r="G103" s="2">
-        <v>57</v>
+        <v>1121</v>
       </c>
       <c r="H103" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="104" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="104" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C104" s="2" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="F104" s="8"/>
     </row>
-    <row r="105" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D105" s="2" t="s">
-        <v>1291</v>
-      </c>
-      <c r="E105" s="2">
-        <v>121219</v>
+        <v>1817</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>1818</v>
       </c>
       <c r="F105" s="8"/>
       <c r="G105" s="2">
-        <v>4530</v>
+        <v>1241</v>
       </c>
       <c r="H105" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D106" s="2" t="s">
-        <v>1292</v>
-      </c>
-      <c r="E106" s="2">
-        <v>121082</v>
+        <v>1819</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>1820</v>
       </c>
       <c r="F106" s="8"/>
       <c r="G106" s="2">
-        <v>2287</v>
+        <v>496</v>
       </c>
       <c r="H106" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="107" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="C107" s="2" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F107" s="8"/>
     </row>
-    <row r="108" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
       <c r="D108" s="2" t="s">
-        <v>1337</v>
-      </c>
-      <c r="F108" s="8">
-        <v>6221257000023</v>
+        <v>1821</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>1822</v>
+      </c>
+      <c r="F108" s="8"/>
+      <c r="G108" s="2">
+        <v>510</v>
       </c>
       <c r="H108" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="109" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D109" s="2" t="s">
-        <v>1338</v>
-      </c>
-      <c r="F109" s="8">
-        <v>6223007702263</v>
-      </c>
-      <c r="H109" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="110" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D110" s="2" t="s">
-        <v>1339</v>
-      </c>
-      <c r="E110" s="2" t="s">
-        <v>1340</v>
-      </c>
-      <c r="F110" s="8">
-        <v>6223007702249</v>
-      </c>
-      <c r="G110" s="2">
-        <v>230</v>
-      </c>
-      <c r="H110" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="111" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D111" s="2" t="s">
-        <v>1341</v>
-      </c>
-      <c r="E111" s="2" t="s">
-        <v>1342</v>
-      </c>
-      <c r="F111" s="8">
-        <v>6223007702287</v>
-      </c>
-      <c r="G111" s="2">
-        <v>210</v>
-      </c>
-      <c r="H111" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="112" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D112" s="2" t="s">
-        <v>1343</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>1344</v>
-      </c>
-      <c r="F112" s="8">
-        <v>6223007702256</v>
-      </c>
-      <c r="G112" s="2">
-        <v>253</v>
-      </c>
-      <c r="H112" s="2">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="113" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D113" s="2" t="s">
-        <v>1345</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>1346</v>
-      </c>
-      <c r="F113" s="8">
-        <v>6223007702218</v>
-      </c>
-      <c r="G113" s="2">
-        <v>75</v>
-      </c>
-      <c r="H113" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="114" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D114" s="2" t="s">
-        <v>1347</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>1348</v>
-      </c>
-      <c r="F114" s="8">
-        <v>62230007702287</v>
-      </c>
-      <c r="G114" s="2">
-        <v>240</v>
-      </c>
-      <c r="H114" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="115" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D115" s="2" t="s">
-        <v>1349</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>1350</v>
-      </c>
-      <c r="F115" s="8">
-        <v>6223007702225</v>
-      </c>
-      <c r="G115" s="2">
-        <v>110</v>
-      </c>
-      <c r="H115" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="116" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D116" s="2" t="s">
-        <v>1519</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>1520</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="109" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C109" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F109" s="8"/>
+    </row>
+    <row r="110" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="B110" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F110" s="8"/>
+    </row>
+    <row r="111" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="C111" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F111" s="8"/>
+    </row>
+    <row r="112" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="C112" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F112" s="8"/>
+    </row>
+    <row r="113" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="C113" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="F113" s="8"/>
+    </row>
+    <row r="114" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B114" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="F114" s="8"/>
+    </row>
+    <row r="115" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B115" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="F115" s="8"/>
+    </row>
+    <row r="116" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B116" s="2" t="s">
+        <v>514</v>
       </c>
       <c r="F116" s="8"/>
-      <c r="G116" s="2">
-        <v>165</v>
-      </c>
-      <c r="H116" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D117" s="2" t="s">
-        <v>1521</v>
-      </c>
-      <c r="E117" s="2" t="s">
-        <v>1522</v>
-      </c>
-      <c r="F117" s="8">
-        <v>6221257000054</v>
-      </c>
-      <c r="G117" s="2">
-        <v>70</v>
-      </c>
-      <c r="H117" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="118" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D118" s="2" t="s">
-        <v>1523</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>1524</v>
-      </c>
-      <c r="F118" s="8">
-        <v>6221257000085</v>
-      </c>
-      <c r="G118" s="2">
-        <v>131</v>
-      </c>
-      <c r="H118" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="119" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C119" s="2" t="s">
-        <v>881</v>
-      </c>
+    </row>
+    <row r="117" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B117" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="F117" s="8"/>
+    </row>
+    <row r="118" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="F118" s="8"/>
+    </row>
+    <row r="119" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F119" s="8"/>
     </row>
-    <row r="120" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D120" s="2" t="s">
-        <v>1374</v>
-      </c>
-      <c r="E120" s="2" t="s">
-        <v>1375</v>
-      </c>
+    <row r="120" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F120" s="8"/>
-      <c r="G120" s="2">
-        <v>1430</v>
-      </c>
-      <c r="H120" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D121" s="2" t="s">
-        <v>1376</v>
-      </c>
-      <c r="E121" s="2" t="s">
-        <v>1377</v>
-      </c>
+    </row>
+    <row r="121" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F121" s="8"/>
-      <c r="H121" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C122" s="2" t="s">
-        <v>20</v>
-      </c>
+    </row>
+    <row r="122" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F122" s="8"/>
     </row>
-    <row r="123" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C123" s="2" t="s">
-        <v>682</v>
-      </c>
+    <row r="123" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F123" s="8"/>
     </row>
-    <row r="124" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C124" s="2" t="s">
-        <v>22</v>
-      </c>
+    <row r="124" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F124" s="8"/>
     </row>
-    <row r="125" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C125" s="2" t="s">
-        <v>293</v>
-      </c>
+    <row r="125" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F125" s="8"/>
     </row>
-    <row r="126" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C126" s="2" t="s">
-        <v>1300</v>
-      </c>
+    <row r="126" spans="2:6" x14ac:dyDescent="0.3">
       <c r="F126" s="8"/>
     </row>
-    <row r="127" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D127" s="2" t="s">
-        <v>1301</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>1302</v>
-      </c>
-      <c r="F127" s="8" t="s">
-        <v>1303</v>
-      </c>
-      <c r="G127" s="2">
-        <v>211</v>
-      </c>
-      <c r="H127" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="128" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C128" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F128" s="8"/>
-    </row>
-    <row r="129" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D129" s="2" t="s">
-        <v>1462</v>
-      </c>
-      <c r="E129" s="2" t="s">
-        <v>1463</v>
-      </c>
-      <c r="F129" s="8">
-        <v>6221257447316</v>
-      </c>
-      <c r="G129" s="2">
-        <v>125</v>
-      </c>
-      <c r="H129" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="130" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C130" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F130" s="8"/>
-    </row>
-    <row r="131" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D131" s="2" t="s">
-        <v>1482</v>
-      </c>
-      <c r="E131" s="2" t="s">
-        <v>1483</v>
-      </c>
-      <c r="F131" s="8"/>
-      <c r="G131" s="2">
-        <v>20</v>
-      </c>
-      <c r="H131" s="2">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="132" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D132" s="2" t="s">
-        <v>1484</v>
-      </c>
-      <c r="E132" s="2" t="s">
-        <v>1485</v>
-      </c>
-      <c r="F132" s="8">
-        <v>6221257526400</v>
-      </c>
-      <c r="G132" s="2">
-        <v>26</v>
-      </c>
-      <c r="H132" s="2">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="133" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C133" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F133" s="8"/>
-    </row>
-    <row r="134" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D134" s="2" t="s">
-        <v>1366</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>1367</v>
-      </c>
-      <c r="F134" s="8"/>
-      <c r="G134" s="2">
-        <v>910</v>
-      </c>
-      <c r="H134" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D135" s="2" t="s">
-        <v>1368</v>
-      </c>
-      <c r="E135" s="2" t="s">
-        <v>1369</v>
-      </c>
-      <c r="F135" s="8"/>
-      <c r="H135" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D136" s="2" t="s">
-        <v>1370</v>
-      </c>
-      <c r="E136" s="2" t="s">
-        <v>1371</v>
-      </c>
-      <c r="F136" s="8"/>
-      <c r="H136" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D137" s="2" t="s">
-        <v>1372</v>
-      </c>
-      <c r="E137" s="2" t="s">
-        <v>1373</v>
-      </c>
-      <c r="F137" s="8"/>
-      <c r="G137" s="2">
-        <v>950</v>
-      </c>
-      <c r="H137" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C138" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F138" s="8"/>
-    </row>
-    <row r="139" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C139" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="F139" s="8"/>
-    </row>
-    <row r="140" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C140" s="2" t="s">
-        <v>898</v>
-      </c>
-      <c r="F140" s="8"/>
-    </row>
-    <row r="141" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C141" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F141" s="8"/>
-    </row>
-    <row r="142" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D142" s="2" t="s">
-        <v>1509</v>
-      </c>
-      <c r="E142" s="2" t="s">
-        <v>1510</v>
-      </c>
-      <c r="F142" s="8">
-        <v>3800031500</v>
-      </c>
-      <c r="G142" s="2">
-        <v>1086</v>
-      </c>
-      <c r="H142" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="143" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D143" s="2" t="s">
-        <v>1511</v>
-      </c>
-      <c r="E143" s="2" t="s">
-        <v>1512</v>
-      </c>
-      <c r="F143" s="8">
-        <v>6221257441611</v>
-      </c>
-      <c r="G143" s="2">
-        <v>1352</v>
-      </c>
-      <c r="H143" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D144" s="2" t="s">
-        <v>1513</v>
-      </c>
-      <c r="E144" s="2" t="s">
-        <v>1514</v>
-      </c>
-      <c r="F144" s="8">
-        <v>6221257441611</v>
-      </c>
-      <c r="G144" s="2">
-        <v>412</v>
-      </c>
-      <c r="H144" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="145" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D145" s="2" t="s">
-        <v>1515</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>1516</v>
-      </c>
-      <c r="F145" s="8">
-        <v>6221257018509</v>
-      </c>
-      <c r="G145" s="2">
-        <v>493</v>
-      </c>
-      <c r="H145" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="146" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D146" s="2" t="s">
-        <v>1517</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>1518</v>
-      </c>
-      <c r="F146" s="8"/>
-      <c r="G146" s="2">
-        <v>600</v>
-      </c>
-      <c r="H146" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="147" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C147" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F147" s="8"/>
-    </row>
-    <row r="148" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C148" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F148" s="8"/>
-    </row>
-    <row r="149" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D149" s="2" t="s">
-        <v>1405</v>
-      </c>
-      <c r="E149" s="2" t="s">
-        <v>1406</v>
-      </c>
-      <c r="F149" s="8"/>
-      <c r="G149" s="2">
-        <v>135</v>
-      </c>
-      <c r="H149" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D150" s="2" t="s">
-        <v>1407</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>1408</v>
-      </c>
-      <c r="F150" s="8">
-        <v>6221257483871</v>
-      </c>
-      <c r="G150" s="2">
-        <v>450</v>
-      </c>
-      <c r="H150" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="151" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D151" s="2" t="s">
-        <v>1409</v>
-      </c>
-      <c r="E151" s="2" t="s">
-        <v>1410</v>
-      </c>
-      <c r="F151" s="8">
-        <v>6221257375541</v>
-      </c>
-      <c r="G151" s="2">
-        <v>123</v>
-      </c>
-      <c r="H151" s="2">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="152" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D152" s="2" t="s">
-        <v>1490</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>1491</v>
-      </c>
-      <c r="F152" s="8">
-        <v>6221257435290</v>
-      </c>
-      <c r="G152" s="2">
-        <v>148</v>
-      </c>
-      <c r="H152" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="153" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D153" s="2" t="s">
-        <v>1498</v>
-      </c>
-      <c r="E153" s="2">
-        <v>3616</v>
-      </c>
-      <c r="F153" s="8"/>
-      <c r="G153" s="2">
-        <v>168</v>
-      </c>
-      <c r="H153" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="154" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C154" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F154" s="8"/>
-    </row>
-    <row r="155" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C155" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F155" s="8"/>
-    </row>
-    <row r="156" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B156" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F156" s="8"/>
-    </row>
-    <row r="157" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C157" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="F157" s="8"/>
-    </row>
-    <row r="158" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C158" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F158" s="8"/>
-    </row>
-    <row r="159" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C159" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F159" s="8"/>
-    </row>
-    <row r="160" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D160" s="2" t="s">
-        <v>1425</v>
-      </c>
-      <c r="E160" s="2" t="s">
-        <v>1426</v>
-      </c>
-      <c r="F160" s="8"/>
-      <c r="G160" s="2">
-        <v>182</v>
-      </c>
-      <c r="H160" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="161" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D161" s="2" t="s">
-        <v>1427</v>
-      </c>
-      <c r="E161" s="2" t="s">
-        <v>1428</v>
-      </c>
-      <c r="F161" s="8">
-        <v>9605760103124</v>
-      </c>
-      <c r="G161" s="2">
-        <v>357</v>
-      </c>
-      <c r="H161" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="162" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D162" s="2" t="s">
-        <v>1429</v>
-      </c>
-      <c r="E162" s="2" t="s">
-        <v>1430</v>
-      </c>
-      <c r="F162" s="8">
-        <v>9605760102110</v>
-      </c>
-      <c r="G162" s="2">
-        <v>169</v>
-      </c>
-      <c r="H162" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="163" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D163" s="2" t="s">
-        <v>1441</v>
-      </c>
-      <c r="E163" s="2" t="s">
-        <v>1442</v>
-      </c>
-      <c r="F163" s="8"/>
-      <c r="G163" s="2">
-        <v>90</v>
-      </c>
-      <c r="H163" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="164" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D164" s="2" t="s">
-        <v>1443</v>
-      </c>
-      <c r="E164" s="2" t="s">
-        <v>1444</v>
-      </c>
-      <c r="F164" s="8"/>
-      <c r="H164" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="165" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D165" s="2" t="s">
-        <v>1505</v>
-      </c>
-      <c r="E165" s="2" t="s">
-        <v>1506</v>
-      </c>
-      <c r="F165" s="8">
-        <v>6221257031089</v>
-      </c>
-      <c r="G165" s="2">
-        <v>775</v>
-      </c>
-      <c r="H165" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="166" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D166" s="2" t="s">
-        <v>1507</v>
-      </c>
-      <c r="E166" s="2" t="s">
-        <v>1508</v>
-      </c>
-      <c r="F166" s="8">
-        <v>9605760105135</v>
-      </c>
-      <c r="G166" s="2">
-        <v>703</v>
-      </c>
-      <c r="H166" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="167" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C167" s="2" t="s">
-        <v>355</v>
-      </c>
-      <c r="F167" s="8"/>
-    </row>
-    <row r="168" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C168" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F168" s="8"/>
-    </row>
-    <row r="169" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D169" s="2" t="s">
-        <v>1486</v>
-      </c>
-      <c r="E169" s="2" t="s">
-        <v>1487</v>
-      </c>
-      <c r="F169" s="8"/>
-      <c r="G169" s="2">
-        <v>49</v>
-      </c>
-      <c r="H169" s="2">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="170" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D170" s="2" t="s">
-        <v>1488</v>
-      </c>
-      <c r="E170" s="2" t="s">
-        <v>1489</v>
-      </c>
-      <c r="F170" s="8"/>
-      <c r="G170" s="2">
-        <v>11</v>
-      </c>
-      <c r="H170" s="2">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="171" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C171" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="F171" s="8"/>
-    </row>
-    <row r="172" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C172" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F172" s="8"/>
-    </row>
-    <row r="173" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D173" s="2" t="s">
-        <v>1527</v>
-      </c>
-      <c r="E173" s="2" t="s">
-        <v>1528</v>
-      </c>
-      <c r="F173" s="8">
-        <v>6221257466782</v>
-      </c>
-      <c r="G173" s="2">
-        <v>21</v>
-      </c>
-      <c r="H173" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="174" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B174" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="F174" s="8"/>
-    </row>
-    <row r="175" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C175" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="F175" s="8"/>
-    </row>
-    <row r="176" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C176" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="F176" s="8"/>
-    </row>
-    <row r="177" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D177" s="2" t="s">
-        <v>1204</v>
-      </c>
-      <c r="E177" s="2" t="s">
-        <v>1205</v>
-      </c>
-      <c r="F177" s="8">
-        <v>6221257354089</v>
-      </c>
-      <c r="G177" s="2">
-        <v>1363</v>
-      </c>
-      <c r="H177" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="178" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D178" s="2" t="s">
-        <v>1206</v>
-      </c>
-      <c r="E178" s="2" t="s">
-        <v>1207</v>
-      </c>
-      <c r="F178" s="8"/>
-      <c r="G178" s="2">
-        <v>1815</v>
-      </c>
-      <c r="H178" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="179" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D179" s="2" t="s">
-        <v>1208</v>
-      </c>
-      <c r="E179" s="2" t="s">
-        <v>1209</v>
-      </c>
-      <c r="F179" s="8">
-        <v>6221257527667</v>
-      </c>
-      <c r="G179" s="2">
-        <v>1197</v>
-      </c>
-      <c r="H179" s="2">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="180" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D180" s="2" t="s">
-        <v>1210</v>
-      </c>
-      <c r="E180" s="2" t="s">
-        <v>1209</v>
-      </c>
-      <c r="F180" s="8">
-        <v>6221257527667</v>
-      </c>
-      <c r="G180" s="2">
-        <v>1575</v>
-      </c>
-      <c r="H180" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="181" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D181" s="2" t="s">
-        <v>1211</v>
-      </c>
-      <c r="E181" s="2" t="s">
-        <v>1212</v>
-      </c>
-      <c r="F181" s="8">
-        <v>6221257527315</v>
-      </c>
-      <c r="G181" s="2">
-        <v>1290</v>
-      </c>
-      <c r="H181" s="2">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="182" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D182" s="2" t="s">
-        <v>1213</v>
-      </c>
-      <c r="E182" s="2" t="s">
-        <v>1214</v>
-      </c>
-      <c r="F182" s="8">
-        <v>6221257527346</v>
-      </c>
-      <c r="G182" s="2">
-        <v>1938</v>
-      </c>
-      <c r="H182" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="183" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D183" s="2" t="s">
-        <v>1215</v>
-      </c>
-      <c r="E183" s="2" t="s">
-        <v>1216</v>
-      </c>
-      <c r="F183" s="8">
-        <v>6221257523904</v>
-      </c>
-      <c r="G183" s="2">
-        <v>731</v>
-      </c>
-      <c r="H183" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="184" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D184" s="2" t="s">
-        <v>1217</v>
-      </c>
-      <c r="E184" s="2" t="s">
-        <v>1218</v>
-      </c>
-      <c r="F184" s="8">
-        <v>6221257527728</v>
-      </c>
-      <c r="G184" s="2">
-        <v>1800</v>
-      </c>
-      <c r="H184" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="185" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D185" s="2" t="s">
-        <v>1417</v>
-      </c>
-      <c r="E185" s="2" t="s">
-        <v>1418</v>
-      </c>
-      <c r="F185" s="8">
-        <v>6221257527377</v>
-      </c>
-      <c r="G185" s="2">
-        <v>2116</v>
-      </c>
-      <c r="H185" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="186" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C186" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F186" s="8"/>
-    </row>
-    <row r="187" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C187" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F187" s="8"/>
-    </row>
-    <row r="188" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C188" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="F188" s="8"/>
-    </row>
-    <row r="189" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C189" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="F189" s="8"/>
-    </row>
-    <row r="190" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D190" s="2" t="s">
-        <v>1419</v>
-      </c>
-      <c r="E190" s="2" t="s">
-        <v>1420</v>
-      </c>
-      <c r="F190" s="8">
-        <v>6221257527445</v>
-      </c>
-      <c r="G190" s="2">
-        <v>2777</v>
-      </c>
-      <c r="H190" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="191" spans="2:8" ht="17.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C191" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F191" s="8"/>
-    </row>
-    <row r="192" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B192" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F192" s="8"/>
-    </row>
-    <row r="193" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C193" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F193" s="8"/>
-    </row>
-    <row r="194" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C194" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F194" s="8"/>
-    </row>
-    <row r="195" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D195" s="2" t="s">
-        <v>1326</v>
-      </c>
-      <c r="E195" s="2" t="s">
-        <v>1327</v>
-      </c>
-      <c r="F195" s="8"/>
-      <c r="G195" s="2">
-        <v>518</v>
-      </c>
-      <c r="H195" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="196" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D196" s="2" t="s">
-        <v>1328</v>
-      </c>
-      <c r="F196" s="8">
-        <v>6221257483994</v>
-      </c>
-      <c r="G196" s="2">
-        <v>435</v>
-      </c>
-      <c r="H196" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="197" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D197" s="2" t="s">
-        <v>1329</v>
-      </c>
-      <c r="E197" s="2" t="s">
-        <v>1330</v>
-      </c>
-      <c r="F197" s="8">
-        <v>6221257470802</v>
-      </c>
-      <c r="G197" s="2">
-        <v>761</v>
-      </c>
-      <c r="H197" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="198" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D198" s="2" t="s">
-        <v>1331</v>
-      </c>
-      <c r="E198" s="2" t="s">
-        <v>1332</v>
-      </c>
-      <c r="F198" s="8"/>
-      <c r="G198" s="2">
-        <v>1203</v>
-      </c>
-      <c r="H198" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="199" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D199" s="2" t="s">
-        <v>1333</v>
-      </c>
-      <c r="E199" s="2" t="s">
-        <v>1334</v>
-      </c>
-      <c r="F199" s="8">
-        <v>6221257470819</v>
-      </c>
-      <c r="G199" s="2">
-        <v>1521</v>
-      </c>
-      <c r="H199" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="200" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D200" s="2" t="s">
-        <v>1335</v>
-      </c>
-      <c r="E200" s="2" t="s">
-        <v>1336</v>
-      </c>
-      <c r="F200" s="8">
-        <v>6221257470871</v>
-      </c>
-      <c r="G200" s="2">
-        <v>2559</v>
-      </c>
-      <c r="H200" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="201" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C201" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F201" s="8"/>
-    </row>
-    <row r="202" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C202" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="F202" s="8"/>
-    </row>
-    <row r="203" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D203" s="2" t="s">
-        <v>1492</v>
-      </c>
-      <c r="E203" s="2" t="s">
-        <v>1493</v>
-      </c>
-      <c r="F203" s="8">
-        <v>6223007708197</v>
-      </c>
-      <c r="G203" s="2">
-        <v>130</v>
-      </c>
-      <c r="H203" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="204" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D204" s="2" t="s">
-        <v>1494</v>
-      </c>
-      <c r="E204" s="2" t="s">
-        <v>1495</v>
-      </c>
-      <c r="F204" s="8">
-        <v>6223007708203</v>
-      </c>
-      <c r="G204" s="2">
-        <v>201</v>
-      </c>
-      <c r="H204" s="2">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="205" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D205" s="2" t="s">
-        <v>1496</v>
-      </c>
-      <c r="E205" s="2" t="s">
-        <v>1497</v>
-      </c>
-      <c r="F205" s="8">
-        <v>6223007708234</v>
-      </c>
-      <c r="G205" s="2">
-        <v>318</v>
-      </c>
-      <c r="H205" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="206" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C206" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F206" s="8"/>
-    </row>
-    <row r="207" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C207" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F207" s="8"/>
-    </row>
-    <row r="208" spans="3:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D208" s="2" t="s">
-        <v>1431</v>
-      </c>
-      <c r="E208" s="2" t="s">
-        <v>1432</v>
-      </c>
-      <c r="F208" s="8"/>
-      <c r="G208" s="2">
-        <v>5228</v>
-      </c>
-      <c r="H208" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="209" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D209" s="2" t="s">
-        <v>1433</v>
-      </c>
-      <c r="E209" s="2" t="s">
-        <v>1434</v>
-      </c>
-      <c r="F209" s="8">
-        <v>6221257484533</v>
-      </c>
-      <c r="G209" s="2">
-        <v>2642</v>
-      </c>
-      <c r="H209" s="2">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="210" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D210" s="2" t="s">
-        <v>1435</v>
-      </c>
-      <c r="E210" s="2" t="s">
-        <v>1436</v>
-      </c>
-      <c r="F210" s="8"/>
-      <c r="G210" s="2">
-        <v>1992</v>
-      </c>
-      <c r="H210" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="211" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D211" s="2" t="s">
-        <v>1437</v>
-      </c>
-      <c r="E211" s="2" t="s">
-        <v>1438</v>
-      </c>
-      <c r="F211" s="8"/>
-      <c r="G211" s="2">
-        <v>2589</v>
-      </c>
-      <c r="H211" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="212" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D212" s="2" t="s">
-        <v>1439</v>
-      </c>
-      <c r="E212" s="2" t="s">
-        <v>1440</v>
-      </c>
-      <c r="F212" s="8">
-        <v>6221257484557</v>
-      </c>
-      <c r="G212" s="2">
-        <v>3124</v>
-      </c>
-      <c r="H212" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="213" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C213" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F213" s="8"/>
-    </row>
-    <row r="214" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D214" s="2" t="s">
-        <v>1252</v>
-      </c>
-      <c r="E214" s="2" t="s">
-        <v>1253</v>
-      </c>
-      <c r="F214" s="8"/>
-      <c r="G214" s="2">
-        <v>2690</v>
-      </c>
-      <c r="H214" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="215" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B215" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F215" s="8"/>
-    </row>
-    <row r="216" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C216" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F216" s="8"/>
-    </row>
-    <row r="217" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D217" s="2" t="s">
-        <v>1314</v>
-      </c>
-      <c r="E217" s="2" t="s">
-        <v>1315</v>
-      </c>
-      <c r="F217" s="8">
-        <v>6221257470680</v>
-      </c>
-      <c r="G217" s="2">
-        <v>64</v>
-      </c>
-      <c r="H217" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="218" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D218" s="2" t="s">
-        <v>1316</v>
-      </c>
-      <c r="E218" s="2" t="s">
-        <v>1317</v>
-      </c>
-      <c r="F218" s="8">
-        <v>6221257442557</v>
-      </c>
-      <c r="H218" s="2">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="219" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D219" s="2" t="s">
-        <v>1318</v>
-      </c>
-      <c r="E219" s="2" t="s">
-        <v>1319</v>
-      </c>
-      <c r="F219" s="8">
-        <v>6223007702560</v>
-      </c>
-    </row>
-    <row r="220" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D220" s="2" t="s">
-        <v>1320</v>
-      </c>
-      <c r="E220" s="2" t="s">
-        <v>1321</v>
-      </c>
-      <c r="F220" s="8">
-        <v>6221257470697</v>
-      </c>
-      <c r="G220" s="2">
-        <v>97</v>
-      </c>
-      <c r="H220" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="221" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D221" s="2" t="s">
-        <v>1322</v>
-      </c>
-      <c r="E221" s="2" t="s">
-        <v>1323</v>
-      </c>
-      <c r="F221" s="8">
-        <v>6223007702591</v>
-      </c>
-      <c r="G221" s="2">
-        <v>167</v>
-      </c>
-      <c r="H221" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="222" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D222" s="2" t="s">
-        <v>1324</v>
-      </c>
-      <c r="E222" s="2" t="s">
-        <v>1325</v>
-      </c>
-      <c r="F222" s="8">
-        <v>6221257442601</v>
-      </c>
-      <c r="G222" s="2">
-        <v>60</v>
-      </c>
-      <c r="H222" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="223" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C223" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F223" s="8"/>
-    </row>
-    <row r="224" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C224" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F224" s="8"/>
-    </row>
-    <row r="225" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D225" s="2" t="s">
-        <v>1310</v>
-      </c>
-      <c r="E225" s="2" t="s">
-        <v>1311</v>
-      </c>
-      <c r="F225" s="8"/>
-      <c r="G225" s="2">
-        <v>226</v>
-      </c>
-      <c r="H225" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="226" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D226" s="2" t="s">
-        <v>1312</v>
-      </c>
-      <c r="E226" s="2" t="s">
-        <v>1313</v>
-      </c>
-      <c r="F226" s="8">
-        <v>6221257024364</v>
-      </c>
-      <c r="G226" s="2">
-        <v>170</v>
-      </c>
-      <c r="H226" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="227" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C227" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F227" s="8"/>
-    </row>
-    <row r="228" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D228" s="2" t="s">
-        <v>1421</v>
-      </c>
-      <c r="E228" s="2" t="s">
-        <v>1422</v>
-      </c>
-      <c r="F228" s="8">
-        <v>6221257537918</v>
-      </c>
-      <c r="G228" s="2">
-        <v>1898</v>
-      </c>
-      <c r="H228" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="229" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D229" s="2" t="s">
-        <v>1423</v>
-      </c>
-      <c r="E229" s="2" t="s">
-        <v>1424</v>
-      </c>
-      <c r="F229" s="8">
-        <v>6221257537956</v>
-      </c>
-      <c r="G229" s="2">
-        <v>3127</v>
-      </c>
-      <c r="H229" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="230" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D230" s="2" t="s">
-        <v>1415</v>
-      </c>
-      <c r="E230" s="2" t="s">
-        <v>1416</v>
-      </c>
-      <c r="F230" s="8">
-        <v>6221257537970</v>
-      </c>
-      <c r="G230" s="2">
-        <v>361</v>
-      </c>
-      <c r="H230" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="231" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="F231" s="8"/>
-    </row>
-    <row r="232" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C232" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F232" s="8"/>
-    </row>
-    <row r="233" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D233" s="2" t="s">
-        <v>1453</v>
-      </c>
-      <c r="E233" s="2" t="s">
-        <v>1454</v>
-      </c>
-      <c r="F233" s="8">
-        <v>6221257025019</v>
-      </c>
-      <c r="G233" s="2">
-        <v>54</v>
-      </c>
-      <c r="H233" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="234" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D234" s="2" t="s">
-        <v>1455</v>
-      </c>
-      <c r="E234" s="2" t="s">
-        <v>1456</v>
-      </c>
-      <c r="F234" s="8"/>
-      <c r="G234" s="2">
-        <v>54</v>
-      </c>
-      <c r="H234" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="235" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D235" s="2" t="s">
-        <v>1457</v>
-      </c>
-      <c r="E235" s="2" t="s">
-        <v>1458</v>
-      </c>
-      <c r="F235" s="8">
-        <v>6221257025033</v>
-      </c>
-      <c r="G235" s="2">
-        <v>57</v>
-      </c>
-      <c r="H235" s="2">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="236" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="D236" s="2" t="s">
-        <v>1459</v>
-      </c>
-      <c r="E236" s="2" t="s">
-        <v>1460</v>
-      </c>
-      <c r="F236" s="8">
-        <v>6221257025019</v>
-      </c>
-      <c r="G236" s="2">
-        <v>56</v>
-      </c>
-      <c r="H236" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="237" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="B237" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F237" s="8"/>
-    </row>
-    <row r="238" spans="2:8" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="C238" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F238" s="8"/>
-    </row>
-    <row r="239" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C239" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F239" s="8"/>
-    </row>
-    <row r="240" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="C240" s="2" t="s">
-        <v>264</v>
-      </c>
-      <c r="F240" s="8"/>
-    </row>
-    <row r="241" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D241" s="2" t="s">
-        <v>1296</v>
-      </c>
-      <c r="E241" s="2" t="s">
-        <v>1297</v>
-      </c>
-      <c r="F241" s="8">
-        <v>6221257039405</v>
-      </c>
-      <c r="G241" s="2">
-        <v>230</v>
-      </c>
-      <c r="H241" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="242" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D242" s="2" t="s">
-        <v>1298</v>
-      </c>
-      <c r="E242" s="2" t="s">
-        <v>1299</v>
-      </c>
-      <c r="F242" s="8"/>
-      <c r="G242" s="2">
-        <v>90</v>
-      </c>
-      <c r="H242" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="243" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D243" s="2" t="s">
-        <v>1304</v>
-      </c>
-      <c r="E243" s="2" t="s">
-        <v>1305</v>
-      </c>
-      <c r="F243" s="8">
-        <v>6221257038804</v>
-      </c>
-      <c r="G243" s="2">
-        <v>500</v>
-      </c>
-      <c r="H243" s="2">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="244" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D244" s="2" t="s">
-        <v>1306</v>
-      </c>
-      <c r="E244" s="2" t="s">
-        <v>1307</v>
-      </c>
-      <c r="F244" s="8">
-        <v>6221257038750</v>
-      </c>
-      <c r="G244" s="2">
-        <v>860</v>
-      </c>
-      <c r="H244" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="245" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D245" s="2" t="s">
-        <v>1308</v>
-      </c>
-      <c r="E245" s="2" t="s">
-        <v>1309</v>
-      </c>
-      <c r="F245" s="8">
-        <v>6221257038804</v>
-      </c>
-      <c r="G245" s="2">
-        <v>787</v>
-      </c>
-      <c r="H245" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="246" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D246" s="2" t="s">
-        <v>1476</v>
-      </c>
-      <c r="E246" s="2" t="s">
-        <v>1477</v>
-      </c>
-      <c r="F246" s="8">
-        <v>6221257038705</v>
-      </c>
-      <c r="G246" s="2">
-        <v>905</v>
-      </c>
-      <c r="H246" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="247" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D247" s="2" t="s">
-        <v>1478</v>
-      </c>
-      <c r="E247" s="2" t="s">
-        <v>1479</v>
-      </c>
-      <c r="F247" s="8"/>
-      <c r="G247" s="2">
-        <v>590</v>
-      </c>
-      <c r="H247" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="248" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="D248" s="2" t="s">
-        <v>1499</v>
-      </c>
-      <c r="E248" s="2" t="s">
-        <v>1500</v>
-      </c>
-      <c r="F248" s="8">
-        <v>6221257001945</v>
-      </c>
-      <c r="G248" s="2">
-        <v>3525</v>
-      </c>
-      <c r="H248" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="249" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B249" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="F249" s="8"/>
-    </row>
-    <row r="250" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B250" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="F250" s="8"/>
-    </row>
-    <row r="251" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B251" s="2" t="s">
-        <v>514</v>
-      </c>
-      <c r="F251" s="8"/>
-    </row>
-    <row r="252" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B252" s="2" t="s">
-        <v>705</v>
-      </c>
-      <c r="F252" s="8"/>
-    </row>
-    <row r="253" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="F253" s="8"/>
-    </row>
-    <row r="257" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F257" s="8"/>
-    </row>
-    <row r="258" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F258" s="8"/>
-    </row>
-    <row r="259" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F259" s="8"/>
-    </row>
-    <row r="260" spans="6:6" x14ac:dyDescent="0.3">
-      <c r="F260" s="8"/>
+    <row r="127" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="F127" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>